<commit_message>
#5 eSpark BOM Added.
</commit_message>
<xml_diff>
--- a/Design_files/Control_Board/Deliverables/BOM/Client BOM.xlsx
+++ b/Design_files/Control_Board/Deliverables/BOM/Client BOM.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26924"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\eSpark-Consultants\elijahkorp-controlproject\Design_files\Control_Board\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\elijahkorp-controlproject\Design_files\Control_Board\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF13EE2F-96FE-4F26-A620-4E71710C752C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
     <sheet name="10 Boards" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -32,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="551" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="198">
   <si>
     <t>Component list</t>
   </si>
@@ -590,15 +589,6 @@
     <t>Aliexpress</t>
   </si>
   <si>
-    <t>LithiumIonBatteries ROHS</t>
-  </si>
-  <si>
-    <t>maxell CR2032</t>
-  </si>
-  <si>
-    <t>Maxell</t>
-  </si>
-  <si>
     <t>LCSC</t>
   </si>
   <si>
@@ -618,14 +608,32 @@
   </si>
   <si>
     <t>Mainstream Performance line, Arm</t>
+  </si>
+  <si>
+    <t>19mm Waterproof Momentary Latching Metal Doorbell Bell Horn Push Button Switch LED Ring Mark Fixation 5V 12V 24V 220 Lock Reset</t>
+  </si>
+  <si>
+    <t>White LED Button</t>
+  </si>
+  <si>
+    <t>Red LED Button</t>
+  </si>
+  <si>
+    <t>Original For Panasonic CR2032 CR 2032 DL2032 ECR2032 Lithium Battery Watch Calculator Car Key Remote Control Button Coin Cells</t>
+  </si>
+  <si>
+    <t>CR2032</t>
+  </si>
+  <si>
+    <t>Panasonic</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
+    <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -639,21 +647,21 @@
       <sz val="10"/>
       <color indexed="13"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="24"/>
       <color indexed="10"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="24"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -661,7 +669,7 @@
       <sz val="12"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -669,21 +677,21 @@
       <sz val="12"/>
       <color theme="0"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color indexed="10"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -691,71 +699,71 @@
       <sz val="10"/>
       <color theme="0"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="0"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <color indexed="10"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
       <color theme="0"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color indexed="10"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -763,6 +771,7 @@
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -1072,7 +1081,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1570,9 +1579,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:M47"/>
+  <dimension ref="A1:M49"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="57" customWidth="1"/>
@@ -1767,7 +1776,7 @@
     <row r="10" spans="1:13" ht="24">
       <c r="A10" s="2"/>
       <c r="B10" s="34">
-        <f t="shared" ref="B10:B41" si="0">ROW(B10)-ROW($B$9)</f>
+        <f t="shared" ref="B10:B43" si="0">ROW(B10)-ROW($B$9)</f>
         <v>1</v>
       </c>
       <c r="C10" s="35" t="s">
@@ -1795,7 +1804,7 @@
         <v>8</v>
       </c>
       <c r="K10" s="37">
-        <f t="shared" ref="K10:K41" si="1">J10*5</f>
+        <f t="shared" ref="K10:K43" si="1">J10*5</f>
         <v>40</v>
       </c>
       <c r="L10" s="36"/>
@@ -2909,7 +2918,7 @@
       <c r="L40" s="36"/>
       <c r="M40" s="36"/>
     </row>
-    <row r="41" spans="1:13" ht="24">
+    <row r="41" spans="1:13" ht="24.75" thickBot="1">
       <c r="A41" s="2"/>
       <c r="B41" s="34">
         <f t="shared" si="0"/>
@@ -2946,10 +2955,10 @@
       <c r="L41" s="38"/>
       <c r="M41" s="38"/>
     </row>
-    <row r="42" spans="1:13" ht="48">
-      <c r="A42" s="2"/>
+    <row r="42" spans="1:13" s="1" customFormat="1" ht="48.75" thickBot="1">
+      <c r="A42" s="33"/>
       <c r="B42" s="34">
-        <f>ROW(B42)-ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="C42" s="40" t="s">
@@ -2959,36 +2968,34 @@
         <v>55</v>
       </c>
       <c r="E42" s="39" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="F42" s="36" t="s">
         <v>55</v>
       </c>
       <c r="G42" s="38" t="s">
-        <v>55</v>
+        <v>193</v>
       </c>
       <c r="H42" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="I42" s="39" t="s">
-        <v>55</v>
-      </c>
+      <c r="I42" s="39"/>
       <c r="J42" s="38">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K42" s="39">
-        <f>J42*5</f>
-        <v>5</v>
+        <f t="shared" si="1"/>
+        <v>15</v>
       </c>
       <c r="L42" s="54" t="s">
         <v>184</v>
       </c>
       <c r="M42" s="38"/>
     </row>
-    <row r="43" spans="1:13">
-      <c r="A43" s="2"/>
+    <row r="43" spans="1:13" s="1" customFormat="1" ht="48.75" thickBot="1">
+      <c r="A43" s="33"/>
       <c r="B43" s="34">
-        <f>ROW(B43)-ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>34</v>
       </c>
       <c r="C43" s="40" t="s">
@@ -2998,33 +3005,31 @@
         <v>55</v>
       </c>
       <c r="E43" s="39" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="F43" s="36" t="s">
         <v>55</v>
       </c>
       <c r="G43" s="38" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="H43" s="38" t="s">
-        <v>187</v>
-      </c>
-      <c r="I43" s="39" t="s">
-        <v>55</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="I43" s="39"/>
       <c r="J43" s="38">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K43" s="39">
-        <f>J43*5</f>
-        <v>5</v>
+        <f t="shared" si="1"/>
+        <v>10</v>
       </c>
       <c r="L43" s="54" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="M43" s="38"/>
     </row>
-    <row r="44" spans="1:13">
+    <row r="44" spans="1:13" ht="48.75" thickBot="1">
       <c r="A44" s="2"/>
       <c r="B44" s="34">
         <f>ROW(B44)-ROW($B$9)</f>
@@ -3037,16 +3042,16 @@
         <v>55</v>
       </c>
       <c r="E44" s="39" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="F44" s="36" t="s">
         <v>55</v>
       </c>
       <c r="G44" s="38" t="s">
-        <v>190</v>
+        <v>55</v>
       </c>
       <c r="H44" s="38" t="s">
-        <v>191</v>
+        <v>55</v>
       </c>
       <c r="I44" s="39" t="s">
         <v>55</v>
@@ -3059,7 +3064,7 @@
         <v>5</v>
       </c>
       <c r="L44" s="54" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="M44" s="38"/>
     </row>
@@ -3076,18 +3081,18 @@
         <v>55</v>
       </c>
       <c r="E45" s="39" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="F45" s="36" t="s">
         <v>55</v>
       </c>
       <c r="G45" s="38" t="s">
-        <v>55</v>
+        <v>196</v>
       </c>
       <c r="H45" s="38" t="s">
-        <v>55</v>
-      </c>
-      <c r="I45" s="39" t="s">
+        <v>197</v>
+      </c>
+      <c r="I45" s="38" t="s">
         <v>55</v>
       </c>
       <c r="J45" s="38">
@@ -3104,33 +3109,111 @@
     </row>
     <row r="46" spans="1:13">
       <c r="A46" s="2"/>
-      <c r="B46" s="41"/>
-      <c r="C46" s="42"/>
-      <c r="D46" s="43"/>
-      <c r="E46" s="44"/>
-      <c r="F46" s="45"/>
-      <c r="G46" s="46"/>
-      <c r="H46" s="45"/>
-      <c r="I46" s="46"/>
-      <c r="J46" s="46"/>
-      <c r="K46" s="46"/>
-      <c r="L46" s="46"/>
-      <c r="M46" s="55"/>
-    </row>
-    <row r="47" spans="1:13">
+      <c r="B46" s="34">
+        <f>ROW(B46)-ROW($B$9)</f>
+        <v>37</v>
+      </c>
+      <c r="C46" s="40" t="s">
+        <v>182</v>
+      </c>
+      <c r="D46" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="E46" s="39" t="s">
+        <v>186</v>
+      </c>
+      <c r="F46" s="36" t="s">
+        <v>55</v>
+      </c>
+      <c r="G46" s="38" t="s">
+        <v>187</v>
+      </c>
+      <c r="H46" s="38" t="s">
+        <v>188</v>
+      </c>
+      <c r="I46" s="39" t="s">
+        <v>55</v>
+      </c>
+      <c r="J46" s="38">
+        <v>1</v>
+      </c>
+      <c r="K46" s="39">
+        <f>J46*5</f>
+        <v>5</v>
+      </c>
+      <c r="L46" s="54" t="s">
+        <v>185</v>
+      </c>
+      <c r="M46" s="38"/>
+    </row>
+    <row r="47" spans="1:13" ht="48">
       <c r="A47" s="2"/>
-      <c r="B47" s="47"/>
-      <c r="C47" s="48"/>
-      <c r="D47" s="49"/>
-      <c r="E47" s="50"/>
-      <c r="F47" s="50"/>
-      <c r="G47" s="50"/>
-      <c r="H47" s="50"/>
-      <c r="I47" s="50"/>
-      <c r="J47" s="50"/>
-      <c r="K47" s="50"/>
-      <c r="L47" s="50"/>
-      <c r="M47" s="56"/>
+      <c r="B47" s="34">
+        <f>ROW(B47)-ROW($B$9)</f>
+        <v>38</v>
+      </c>
+      <c r="C47" s="40" t="s">
+        <v>182</v>
+      </c>
+      <c r="D47" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="E47" s="39" t="s">
+        <v>189</v>
+      </c>
+      <c r="F47" s="36" t="s">
+        <v>55</v>
+      </c>
+      <c r="G47" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="H47" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="I47" s="39" t="s">
+        <v>55</v>
+      </c>
+      <c r="J47" s="38">
+        <v>1</v>
+      </c>
+      <c r="K47" s="39">
+        <f>J47*5</f>
+        <v>5</v>
+      </c>
+      <c r="L47" s="54" t="s">
+        <v>184</v>
+      </c>
+      <c r="M47" s="38"/>
+    </row>
+    <row r="48" spans="1:13">
+      <c r="A48" s="2"/>
+      <c r="B48" s="41"/>
+      <c r="C48" s="42"/>
+      <c r="D48" s="43"/>
+      <c r="E48" s="44"/>
+      <c r="F48" s="45"/>
+      <c r="G48" s="46"/>
+      <c r="H48" s="45"/>
+      <c r="I48" s="46"/>
+      <c r="J48" s="46"/>
+      <c r="K48" s="46"/>
+      <c r="L48" s="46"/>
+      <c r="M48" s="55"/>
+    </row>
+    <row r="49" spans="1:13">
+      <c r="A49" s="2"/>
+      <c r="B49" s="47"/>
+      <c r="C49" s="48"/>
+      <c r="D49" s="49"/>
+      <c r="E49" s="50"/>
+      <c r="F49" s="50"/>
+      <c r="G49" s="50"/>
+      <c r="H49" s="50"/>
+      <c r="I49" s="50"/>
+      <c r="J49" s="50"/>
+      <c r="K49" s="50"/>
+      <c r="L49" s="50"/>
+      <c r="M49" s="56"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3138,20 +3221,22 @@
     <mergeCell ref="M3:M8"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="L42" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="L43" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="L44" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="L45" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="L44" r:id="rId1"/>
+    <hyperlink ref="L46" r:id="rId2"/>
+    <hyperlink ref="L47" r:id="rId3"/>
+    <hyperlink ref="L42" r:id="rId4"/>
+    <hyperlink ref="L43" r:id="rId5"/>
+    <hyperlink ref="L45" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <drawing r:id="rId5"/>
+  <drawing r:id="rId7"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M47"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:M49"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="3.7109375" customWidth="1"/>
@@ -3345,7 +3430,7 @@
     <row r="10" spans="1:13" s="1" customFormat="1" ht="24">
       <c r="A10" s="33"/>
       <c r="B10" s="34">
-        <f t="shared" ref="B10:B45" si="0">ROW(B10)-ROW($B$9)</f>
+        <f t="shared" ref="B10:B47" si="0">ROW(B10)-ROW($B$9)</f>
         <v>1</v>
       </c>
       <c r="C10" s="35" t="s">
@@ -3410,7 +3495,7 @@
         <v>2</v>
       </c>
       <c r="K11" s="38">
-        <f t="shared" ref="K11:K45" si="1">J11*10</f>
+        <f t="shared" ref="K11:K47" si="1">J11*10</f>
         <v>20</v>
       </c>
       <c r="L11" s="37"/>
@@ -4354,7 +4439,7 @@
         <v>156</v>
       </c>
       <c r="E37" s="39" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="F37" s="38" t="s">
         <v>158</v>
@@ -4428,7 +4513,7 @@
         <v>166</v>
       </c>
       <c r="E39" s="39" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="F39" s="38" t="s">
         <v>168</v>
@@ -4489,7 +4574,7 @@
       <c r="L40" s="37"/>
       <c r="M40" s="36"/>
     </row>
-    <row r="41" spans="1:13" s="1" customFormat="1" ht="24">
+    <row r="41" spans="1:13" s="1" customFormat="1" ht="24.75" thickBot="1">
       <c r="A41" s="33"/>
       <c r="B41" s="34">
         <f t="shared" si="0"/>
@@ -4526,8 +4611,8 @@
       <c r="L41" s="37"/>
       <c r="M41" s="38"/>
     </row>
-    <row r="42" spans="1:13" ht="48">
-      <c r="A42" s="2"/>
+    <row r="42" spans="1:13" s="1" customFormat="1" ht="48.75" thickBot="1">
+      <c r="A42" s="33"/>
       <c r="B42" s="34">
         <f t="shared" si="0"/>
         <v>33</v>
@@ -4539,34 +4624,32 @@
         <v>55</v>
       </c>
       <c r="E42" s="39" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="F42" s="36" t="s">
         <v>55</v>
       </c>
       <c r="G42" s="38" t="s">
-        <v>55</v>
+        <v>193</v>
       </c>
       <c r="H42" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="I42" s="39" t="s">
-        <v>55</v>
-      </c>
+      <c r="I42" s="39"/>
       <c r="J42" s="38">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K42" s="36">
         <f t="shared" si="1"/>
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="L42" s="54" t="s">
         <v>184</v>
       </c>
       <c r="M42" s="38"/>
     </row>
-    <row r="43" spans="1:13">
-      <c r="A43" s="2"/>
+    <row r="43" spans="1:13" s="1" customFormat="1" ht="48.75" thickBot="1">
+      <c r="A43" s="33"/>
       <c r="B43" s="34">
         <f t="shared" si="0"/>
         <v>34</v>
@@ -4578,33 +4661,31 @@
         <v>55</v>
       </c>
       <c r="E43" s="39" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="F43" s="36" t="s">
         <v>55</v>
       </c>
       <c r="G43" s="38" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="H43" s="38" t="s">
-        <v>187</v>
-      </c>
-      <c r="I43" s="39" t="s">
-        <v>55</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="I43" s="39"/>
       <c r="J43" s="38">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K43" s="36">
         <f t="shared" si="1"/>
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="L43" s="54" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="M43" s="38"/>
     </row>
-    <row r="44" spans="1:13">
+    <row r="44" spans="1:13" ht="48.75" thickBot="1">
       <c r="A44" s="2"/>
       <c r="B44" s="34">
         <f t="shared" si="0"/>
@@ -4617,16 +4698,16 @@
         <v>55</v>
       </c>
       <c r="E44" s="39" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="F44" s="36" t="s">
         <v>55</v>
       </c>
       <c r="G44" s="38" t="s">
-        <v>190</v>
+        <v>55</v>
       </c>
       <c r="H44" s="38" t="s">
-        <v>191</v>
+        <v>55</v>
       </c>
       <c r="I44" s="39" t="s">
         <v>55</v>
@@ -4639,7 +4720,7 @@
         <v>10</v>
       </c>
       <c r="L44" s="54" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="M44" s="38"/>
     </row>
@@ -4656,18 +4737,18 @@
         <v>55</v>
       </c>
       <c r="E45" s="39" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="F45" s="36" t="s">
         <v>55</v>
       </c>
       <c r="G45" s="38" t="s">
-        <v>55</v>
+        <v>196</v>
       </c>
       <c r="H45" s="38" t="s">
-        <v>55</v>
-      </c>
-      <c r="I45" s="39" t="s">
+        <v>197</v>
+      </c>
+      <c r="I45" s="38" t="s">
         <v>55</v>
       </c>
       <c r="J45" s="38">
@@ -4684,33 +4765,111 @@
     </row>
     <row r="46" spans="1:13">
       <c r="A46" s="2"/>
-      <c r="B46" s="41"/>
-      <c r="C46" s="42"/>
-      <c r="D46" s="43"/>
-      <c r="E46" s="44"/>
-      <c r="F46" s="45"/>
-      <c r="G46" s="46"/>
-      <c r="H46" s="45"/>
-      <c r="I46" s="46"/>
-      <c r="J46" s="46"/>
-      <c r="K46" s="46"/>
-      <c r="L46" s="46"/>
-      <c r="M46" s="55"/>
-    </row>
-    <row r="47" spans="1:13">
+      <c r="B46" s="34">
+        <f t="shared" si="0"/>
+        <v>37</v>
+      </c>
+      <c r="C46" s="40" t="s">
+        <v>182</v>
+      </c>
+      <c r="D46" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="E46" s="39" t="s">
+        <v>186</v>
+      </c>
+      <c r="F46" s="36" t="s">
+        <v>55</v>
+      </c>
+      <c r="G46" s="38" t="s">
+        <v>187</v>
+      </c>
+      <c r="H46" s="38" t="s">
+        <v>188</v>
+      </c>
+      <c r="I46" s="39" t="s">
+        <v>55</v>
+      </c>
+      <c r="J46" s="38">
+        <v>1</v>
+      </c>
+      <c r="K46" s="36">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="L46" s="54" t="s">
+        <v>185</v>
+      </c>
+      <c r="M46" s="38"/>
+    </row>
+    <row r="47" spans="1:13" ht="48">
       <c r="A47" s="2"/>
-      <c r="B47" s="47"/>
-      <c r="C47" s="48"/>
-      <c r="D47" s="49"/>
-      <c r="E47" s="50"/>
-      <c r="F47" s="50"/>
-      <c r="G47" s="50"/>
-      <c r="H47" s="50"/>
-      <c r="I47" s="50"/>
-      <c r="J47" s="50"/>
-      <c r="K47" s="50"/>
-      <c r="L47" s="50"/>
-      <c r="M47" s="56"/>
+      <c r="B47" s="34">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+      <c r="C47" s="40" t="s">
+        <v>182</v>
+      </c>
+      <c r="D47" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="E47" s="39" t="s">
+        <v>189</v>
+      </c>
+      <c r="F47" s="36" t="s">
+        <v>55</v>
+      </c>
+      <c r="G47" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="H47" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="I47" s="39" t="s">
+        <v>55</v>
+      </c>
+      <c r="J47" s="38">
+        <v>1</v>
+      </c>
+      <c r="K47" s="36">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="L47" s="54" t="s">
+        <v>184</v>
+      </c>
+      <c r="M47" s="38"/>
+    </row>
+    <row r="48" spans="1:13">
+      <c r="A48" s="2"/>
+      <c r="B48" s="41"/>
+      <c r="C48" s="42"/>
+      <c r="D48" s="43"/>
+      <c r="E48" s="44"/>
+      <c r="F48" s="45"/>
+      <c r="G48" s="46"/>
+      <c r="H48" s="45"/>
+      <c r="I48" s="46"/>
+      <c r="J48" s="46"/>
+      <c r="K48" s="46"/>
+      <c r="L48" s="46"/>
+      <c r="M48" s="55"/>
+    </row>
+    <row r="49" spans="1:13">
+      <c r="A49" s="2"/>
+      <c r="B49" s="47"/>
+      <c r="C49" s="48"/>
+      <c r="D49" s="49"/>
+      <c r="E49" s="50"/>
+      <c r="F49" s="50"/>
+      <c r="G49" s="50"/>
+      <c r="H49" s="50"/>
+      <c r="I49" s="50"/>
+      <c r="J49" s="50"/>
+      <c r="K49" s="50"/>
+      <c r="L49" s="50"/>
+      <c r="M49" s="56"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4718,12 +4877,14 @@
     <mergeCell ref="M3:M8"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="L42" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
-    <hyperlink ref="L43" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
-    <hyperlink ref="L44" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
-    <hyperlink ref="L45" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
+    <hyperlink ref="L44" r:id="rId1"/>
+    <hyperlink ref="L46" r:id="rId2"/>
+    <hyperlink ref="L47" r:id="rId3"/>
+    <hyperlink ref="L42" r:id="rId4"/>
+    <hyperlink ref="L43" r:id="rId5"/>
+    <hyperlink ref="L45" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing r:id="rId5"/>
+  <drawing r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>